<commit_message>
Rewrite Sugar News 2026-09-02
</commit_message>
<xml_diff>
--- a/reports/2026/09/Sugar News 2026-09-02.xlsx
+++ b/reports/2026/09/Sugar News 2026-09-02.xlsx
@@ -505,7 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="118.05" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -513,16 +513,16 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度现货市场显示食糖价格，食糖价格为10天。印度食糖价格仅披露当前水平，缺少前期比较时不单独改变供需方向判断。来源：ChiniMandi（https://www.chinimandi.com/isma-nfcsf-say-no-sugar-shortage-expect-prices-to-ease-in-7-10-days/）。影响：中性</t>
+          <t>ISMA与NFCSF联合表示印度没有食糖短缺，主产区出厂价已回落至₹5,000/公担以下，其中马哈拉施特拉邦S级糖₹4,460-4,500/公担、古吉拉特邦M级糖₹4,740/公担、卡纳塔克邦约₹4,960/公担，部分市场零售价仍约₹63/kg，协会预计7-10天内向₹50-52/kg回落。印度政府已允许精炼糖厂在10月5日前向国内销售约35万吨食糖，TRQ进口申请约80万吨且剩余20万吨申请窗口继续开放，叠加8月225万吨销售配额已售约90%，这些增供和去恐慌措施会增加国内流通糖源并压制节前补库价格。来源：ChiniMandi（https://www.chinimandi.com/isma-nfcsf-say-no-sugar-shortage-expect-prices-to-ease-in-7-10-days/）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>中性：印度食糖价格仅披露当前水平，缺少前期比较时不单独改变供需方向判断。</t>
+          <t>利空：ISMA、NFCSF和印度政府释放出厂价回落、精炼糖入市、TRQ进口和月度配额执行等信号，短期增加印度国内可流通糖源并压制节前采购价格。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="116.95" customHeight="1" s="2">
+    <row r="3" ht="103.2" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>泰国</t>
@@ -530,12 +530,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>泰国气象局预报（2026-09-02），那空沙旺、彭世洛、北碧等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
+          <t>泰国气象局9月2日预报，那空沙旺、彭世洛、北碧等甘蔗主产区有雷阵雨，并可能出现局地大雨。泰国甘蔗仍处于生长期，上述产区降雨补充土壤水分、改善甘蔗生长条件，提高后期甘蔗和食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
+          <t>利空：泰国主产区生长期雷阵雨和局地大雨改善墒情，提升后期甘蔗单产和食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>

</xml_diff>